<commit_message>
Agregar nueva propiedad: Lope de Vega 324, Polanco, CDMX. 65,000 MXN/mes, 2 recamaras, 2.5 banos, 2 estacionamientos, 194 m2, 5 huespedes max, pet friendly, sin balcon, sin amenidades especiales. 9 fotos comprimidas a webp (9.88MB -> 1.02MB) mas thumbnail de portada. Sin resenas por ser propiedad nueva, consistente con el resto de propiedades sin historial de huespedes.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -1304,7 +1304,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1314,42 +1314,42 @@
           <t>Blas Pascal 190, Polanco I Sección, Miguel Hidalgo, 11510 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="0" t="n">
         <v>68000</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="0" t="n">
         <v>3.5</v>
       </c>
-      <c r="F22" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" t="n">
+      <c r="F22" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="0" t="inlineStr">
         <is>
           <t>Terraza, Bodega, Cisterna</t>
         </is>
       </c>
-      <c r="I22" t="n">
+      <c r="I22" s="0" t="n">
         <v>156</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
+      <c r="J22" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K22" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1359,42 +1359,42 @@
           <t>Av. Homero 1516, Polanco II Sección, Miguel Hidalgo, 11530 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="0" t="n">
         <v>66300</v>
       </c>
-      <c r="D23" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="n">
+      <c r="D23" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="0" t="inlineStr">
         <is>
           <t>Balcón, Terraza</t>
         </is>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" s="0" t="n">
         <v>136</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
+      <c r="J23" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K23" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1404,42 +1404,42 @@
           <t>C. Arquímedes 145, Polanco IV Sección, Miguel Hidalgo, 11560 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="0" t="n">
         <v>66300</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E24" s="0" t="n">
         <v>2.5</v>
       </c>
-      <c r="F24" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" t="n">
+      <c r="F24" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="0" t="inlineStr">
         <is>
           <t>Balcón, Roof garden, Terraza, Parrilla, Alberca, Gimnasio</t>
         </is>
       </c>
-      <c r="I24" t="n">
+      <c r="I24" s="0" t="n">
         <v>155</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
+      <c r="J24" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K24" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1449,42 +1449,42 @@
           <t>Córdoba 45, Roma Norte, Cuauhtémoc, 06700 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="0" t="n">
         <v>51000</v>
       </c>
-      <c r="D25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="n">
+      <c r="D25" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="0" t="inlineStr">
         <is>
           <t>Balcón</t>
         </is>
       </c>
-      <c r="I25" t="n">
+      <c r="I25" s="0" t="n">
         <v>112</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
+      <c r="J25" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K25" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1494,42 +1494,42 @@
           <t>Chicontepec 57, Hipódromo Condesa, Cuauhtémoc, 06170 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" s="0" t="n">
         <v>40000</v>
       </c>
-      <c r="D26" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" t="n">
+      <c r="D26" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="0" t="inlineStr">
         <is>
           <t>Balcón, Terraza, Roof garden, Parrilla, Alberca, Gimnasio, Jacuzzi, Spa</t>
         </is>
       </c>
-      <c r="I26" t="n">
+      <c r="I26" s="0" t="n">
         <v>102</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
+      <c r="J26" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K26" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1539,42 +1539,42 @@
           <t>Córdoba 48, Roma Norte, Cuauhtémoc, 06700 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" s="0" t="n">
         <v>51000</v>
       </c>
-      <c r="D27" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="n">
+      <c r="D27" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="I27" t="n">
+      <c r="I27" s="0" t="n">
         <v>115</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1584,42 +1584,42 @@
           <t>Tlaxcala 173, Colonia Condesa, Cuauhtémoc, 06140 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" s="0" t="n">
         <v>30000</v>
       </c>
-      <c r="D28" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" t="n">
+      <c r="D28" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="0" t="inlineStr">
         <is>
           <t>Roof garden, Gimnasio</t>
         </is>
       </c>
-      <c r="I28" t="n">
+      <c r="I28" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J28" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K28" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1629,42 +1629,42 @@
           <t>Praga 14, Juárez, Cuauhtémoc, 06600 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" s="0" t="n">
         <v>25000</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G29" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" t="inlineStr">
+      <c r="G29" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="0" t="inlineStr">
         <is>
           <t>Balcón, Terraza, Roof garden, Gimnasio</t>
         </is>
       </c>
-      <c r="I29" t="n">
+      <c r="I29" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
+      <c r="J29" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K29" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1674,42 +1674,42 @@
           <t>Chicontepec 72, Hipódromo, Cuauhtémoc, 06100 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C30" t="n">
+      <c r="C30" s="0" t="n">
         <v>47000</v>
       </c>
-      <c r="D30" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" t="n">
+      <c r="D30" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="0" t="n">
         <v>2.5</v>
       </c>
-      <c r="F30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" t="n">
+      <c r="F30" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="0" t="inlineStr">
         <is>
           <t>Balcón, Terraza, Gimnasio, Jacuzzi</t>
         </is>
       </c>
-      <c r="I30" t="n">
+      <c r="I30" s="0" t="n">
         <v>143</v>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
+      <c r="J30" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K30" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1719,42 +1719,42 @@
           <t>Sinaloa 186, Roma Norte, Cuauhtémoc, 06700 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" s="0" t="n">
         <v>25000</v>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G31" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" t="inlineStr">
+      <c r="G31" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="0" t="inlineStr">
         <is>
           <t>Balcón, Terraza, Roof garden, Alberca, Gimnasio, Jacuzzi</t>
         </is>
       </c>
-      <c r="I31" t="n">
+      <c r="I31" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
+      <c r="J31" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K31" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1764,42 +1764,42 @@
           <t>Juan de la Barrera 36, Colonia Condesa, Cuauhtémoc, 06140 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" s="0" t="n">
         <v>60000</v>
       </c>
-      <c r="D32" t="n">
-        <v>2</v>
-      </c>
-      <c r="E32" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" t="n">
+      <c r="D32" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G32" t="n">
+      <c r="G32" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H32" s="0" t="inlineStr">
         <is>
           <t>Balcón, Terraza, Roof garden, Parrilla</t>
         </is>
       </c>
-      <c r="I32" t="n">
+      <c r="I32" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
+      <c r="J32" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K32" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1809,42 +1809,42 @@
           <t>Av. Chapultepec 447, Juárez, Cuauhtémoc, 06600 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C33" t="n">
+      <c r="C33" s="0" t="n">
         <v>38000</v>
       </c>
-      <c r="D33" t="n">
-        <v>2</v>
-      </c>
-      <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="n">
+      <c r="D33" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G33" t="n">
+      <c r="G33" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="0" t="inlineStr">
         <is>
           <t>Balcón, Roof garden, Gimnasio</t>
         </is>
       </c>
-      <c r="I33" t="n">
+      <c r="I33" s="0" t="n">
         <v>95</v>
       </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
+      <c r="J33" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K33" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1854,42 +1854,42 @@
           <t>Av. Nuevo León 104, Colonia Condesa, Cuauhtémoc, 06140 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C34" t="n">
+      <c r="C34" s="0" t="n">
         <v>31000</v>
       </c>
-      <c r="D34" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" t="n">
-        <v>2</v>
-      </c>
-      <c r="F34" t="n">
+      <c r="D34" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G34" t="n">
+      <c r="G34" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="0" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="I34" t="n">
+      <c r="I34" s="0" t="n">
         <v>97</v>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1899,42 +1899,79 @@
           <t>C. Querétaro 123, Roma Norte, Cuauhtémoc, 06700 Ciudad de México, CDMX</t>
         </is>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" s="0" t="n">
         <v>22000</v>
       </c>
-      <c r="D35" t="n">
+      <c r="D35" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F35" t="n">
+      <c r="F35" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G35" t="n">
-        <v>2</v>
-      </c>
-      <c r="H35" t="inlineStr">
+      <c r="G35" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" s="0" t="inlineStr">
         <is>
           <t>Balcón, Roof garden</t>
         </is>
       </c>
-      <c r="I35" t="n">
+      <c r="I35" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
+      <c r="J35" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K35" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="4" t="n"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Lope de Vega 324, Polanco, Polanco V Secc, Miguel Hidalgo, 11560 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>65000</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" t="n">
+        <v>5</v>
+      </c>
+      <c r="I36" t="n">
+        <v>194</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="4" t="n"/>

</xml_diff>

<commit_message>
Agregar nueva propiedad: Av Moliere 101, Polanco, CDMX. 71,000 MXN/mes, 2 recamaras, 2.5 banos, 3 estacionamientos, 344 m2, 5 huespedes max, con balcon, pet friendly, amenidades: terraza y roof garden. 10 fotos comprimidas a webp (12.11MB -> 1.06MB) mas thumbnail de portada. Agregada a la lista siempre-disponible. Se corrigio en el proceso un bug real: openpyxl trata value=None en ws.cell() como 'no tocar la celda' en vez de 'vaciarla', lo cual habia sobreescrito por accidente la fila de Lope de Vega y dejado su campo de amenidades con el valor de Moliere. Verificado con la libreria xlsx real del backend antes de subir.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -1934,7 +1934,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -1944,37 +1944,80 @@
           <t>Lope de Vega 324, Polanco, Polanco V Secc, Miguel Hidalgo, 11560 Ciudad de México, CDMX, Mexico</t>
         </is>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" s="0" t="n">
         <v>65000</v>
       </c>
-      <c r="D36" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" t="n">
+      <c r="D36" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="0" t="n">
         <v>2.5</v>
       </c>
-      <c r="F36" t="n">
-        <v>2</v>
-      </c>
-      <c r="G36" t="n">
+      <c r="F36" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="I36" t="n">
+      <c r="H36" s="0" t="n"/>
+      <c r="I36" s="0" t="n">
         <v>194</v>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="0" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K36" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="4" t="n"/>
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Av Moliere 101, Polanco, Polanco III Secc, Miguel Hidalgo, 11540 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="n">
+        <v>71000</v>
+      </c>
+      <c r="D37" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="0" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F37" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="H37" s="0" t="inlineStr">
+        <is>
+          <t>Terraza, Roof garden</t>
+        </is>
+      </c>
+      <c r="I37" s="0" t="n">
+        <v>344</v>
+      </c>
+      <c r="J37" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K37" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="4" t="n"/>

</xml_diff>

<commit_message>
Actualizar precios: Av. Nuevo Leon 104 a 34,000 MXN, Amsterdam 119 a 50,000 MXN, Amsterdam 289 a 44,000 MXN. Verificado con la libreria xlsx real que solo cambio el precio y todos los demas campos quedaron intactos en los 3 archivos.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>40000</v>
+        <v>44000</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>2</v>
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="C21" s="1" t="n">
-        <v>47000</v>
+        <v>50000</v>
       </c>
       <c r="D21" s="1" t="n">
         <v>2</v>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="C34" s="0" t="n">
-        <v>31000</v>
+        <v>34000</v>
       </c>
       <c r="D34" s="0" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Agregar nueva propiedad: Galileo 350, Polanco, CDMX. 51,000 MXN/mes, 2 recamaras, 2.5 banos, 2 estacionamientos, 180 m2, 4 huespedes max, con balcon, pet friendly, amenidad: gym. 12 fotos comprimidas a webp (12.48MB -> 1.26MB) mas thumbnail de portada (comedor, no la fachada). Agregada a la lista siempre-disponible. Nota: se repitio por error el mismo bug de calcular mal la fila destino y se sobreescribio Moliere -- restaurado y verificado con la libreria xlsx real antes de subir, esta vez comprobando las 3 propiedades por nombre, no por posicion.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -2020,7 +2020,49 @@
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="4" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Galileo 350, Polanco, Polanco IV Secc, Miguel Hidalgo, 11550 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>51000</v>
+      </c>
+      <c r="D38" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>180</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="4" t="n"/>

</xml_diff>

<commit_message>
Agregar segunda unidad en el mismo edificio de Hamburgo 32 (unidad distinta a la ya existente): 23,000 MXN/mes, 1 recamara, 1 bano, sin estacionamiento, 44 m2, estudio, 2 huespedes, con balcon, pet friendly negociable, amenidades: terraza, roof garden, gym, jacuzzi, spa, sauna, co-working. 7 fotos comprimidas a webp (8.37MB -> 0.70MB). IMPORTANTE: como comparte la misma direccion que la unidad original de Hamburgo 32, no se pudo usar la lista ALWAYS_AVAILABLE (por texto de direccion, hubiera afectado a ambas) -- se agrego una entrada especifica en FROZEN_AVAILABILITY keyed por CDMX#39 para no tocar la unidad original. Verificado con el servicio real compilado que ambas unidades quedan correctamente diferenciadas.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -2020,7 +2020,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -2030,42 +2030,84 @@
           <t>Galileo 350, Polanco, Polanco IV Secc, Miguel Hidalgo, 11550 Ciudad de México, CDMX, Mexico</t>
         </is>
       </c>
-      <c r="C38" t="n">
+      <c r="C38" s="0" t="n">
         <v>51000</v>
       </c>
-      <c r="D38" t="n">
-        <v>2</v>
-      </c>
-      <c r="E38" t="n">
+      <c r="D38" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" s="0" t="n">
         <v>2.5</v>
       </c>
-      <c r="F38" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" t="n">
+      <c r="F38" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H38" s="0" t="inlineStr">
         <is>
           <t>Gym</t>
         </is>
       </c>
-      <c r="I38" t="n">
+      <c r="I38" s="0" t="n">
         <v>180</v>
       </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
+      <c r="J38" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K38" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="4" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Hamburgo 32, Juárez, Cuauhtémoc, 06600 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>23000</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Terraza, Roof garden, Gym, Jacuzzi, Spa, Sauna, Co-working</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>44</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>negociable</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="4" t="n"/>

</xml_diff>

<commit_message>
Agregar nueva propiedad: Av. P.o de la Reforma 222, Juarez, CDMX (direccion distinta a la ya existente Reforma 150, confirmado antes de agregar). 33,000 MXN/mes, 1 recamara, 1 bano, 1 estacionamiento, 106 m2, 2 huespedes, con balcon, pet friendly, amenidades: terraza, gym, alberca, jacuzzi. Vista panoramica de CDMX en la portada. 10 fotos comprimidas a webp (9.98MB -> 0.98MB). Agregada a la lista siempre-disponible, verificado que no colisiona con Reforma 150. Verificado con el servicio real compilado: 186 propiedades totales, Reforma 150 y todas las adiciones anteriores de esta noche intactas.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -2065,7 +2065,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -2075,42 +2075,84 @@
           <t>Hamburgo 32, Juárez, Cuauhtémoc, 06600 Ciudad de México, CDMX, Mexico</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C39" s="0" t="n">
         <v>23000</v>
       </c>
-      <c r="D39" t="n">
+      <c r="D39" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="G39" t="n">
-        <v>2</v>
-      </c>
-      <c r="H39" t="inlineStr">
+      <c r="G39" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" s="0" t="inlineStr">
         <is>
           <t>Terraza, Roof garden, Gym, Jacuzzi, Spa, Sauna, Co-working</t>
         </is>
       </c>
-      <c r="I39" t="n">
+      <c r="I39" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
+      <c r="J39" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K39" s="0" t="inlineStr">
         <is>
           <t>negociable</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="4" t="n"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Av. P.º de la Reforma 222, Juárez, Cuauhtémoc, 06600 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>33000</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Terraza, Gym, Alberca, Jacuzzi</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>106</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="4" t="n"/>

</xml_diff>

<commit_message>
Agregar nueva propiedad: Av. Baja California 280, Hipodromo, CDMX. 47,000 MXN/mes, 2 recamaras, 2.5 banos, 2 estacionamientos, 112 m2, 4 huespedes, con balcon, pet friendly, amenidad: roof garden. 14 fotos comprimidas a webp (16.62MB -> 1.56MB), con ambos thumbnails de portada generados (sala para shortstaymx, balcon para temporaryrentalsmexico). Agregada a la lista siempre-disponible. Verificado con el servicio real compilado: 187 propiedades totales, todas las adiciones anteriores intactas.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -2110,7 +2110,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -2120,42 +2120,84 @@
           <t>Av. P.º de la Reforma 222, Juárez, Cuauhtémoc, 06600 Ciudad de México, CDMX, Mexico</t>
         </is>
       </c>
-      <c r="C40" t="n">
+      <c r="C40" s="0" t="n">
         <v>33000</v>
       </c>
-      <c r="D40" t="n">
+      <c r="D40" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E40" t="n">
+      <c r="E40" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F40" t="n">
+      <c r="F40" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G40" t="n">
-        <v>2</v>
-      </c>
-      <c r="H40" t="inlineStr">
+      <c r="G40" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" s="0" t="inlineStr">
         <is>
           <t>Terraza, Gym, Alberca, Jacuzzi</t>
         </is>
       </c>
-      <c r="I40" t="n">
+      <c r="I40" s="0" t="n">
         <v>106</v>
       </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
+      <c r="J40" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K40" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="4" t="n"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Av. Baja California 280, Hipódromo, Cuauhtémoc, 06100 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>47000</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" t="n">
+        <v>4</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Roof garden</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>112</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="4" t="n"/>

</xml_diff>

<commit_message>
Add property 42: San Luis Potosi 44
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -2155,7 +2155,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -2165,42 +2165,84 @@
           <t>Av. Baja California 280, Hipódromo, Cuauhtémoc, 06100 Ciudad de México, CDMX, Mexico</t>
         </is>
       </c>
-      <c r="C41" t="n">
+      <c r="C41" s="0" t="n">
         <v>47000</v>
       </c>
-      <c r="D41" t="n">
-        <v>2</v>
-      </c>
-      <c r="E41" t="n">
+      <c r="D41" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="0" t="n">
         <v>2.5</v>
       </c>
-      <c r="F41" t="n">
-        <v>2</v>
-      </c>
-      <c r="G41" t="n">
+      <c r="F41" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="0" t="inlineStr">
         <is>
           <t>Roof garden</t>
         </is>
       </c>
-      <c r="I41" t="n">
+      <c r="I41" s="0" t="n">
         <v>112</v>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
+      <c r="J41" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K41" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="4" t="n"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>San Luis Potosí 44, Roma Nte., Cuauhtémoc, 06700 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>48000</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Terraza, Roof garden, Gym</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>160</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="4" t="n"/>

</xml_diff>

<commit_message>
Agregar propiedad #43: Tennyson 155, Polanco, CDMX. 68,000 MXN/mes, 2 recamaras, 3 banos, 2 estacionamientos, 235 m2, 5 huespedes, sin balcon, pet friendly, amenidades: terraza, jacuzzi. 12 fotos + ambos thumbnails de portada. Agregada a ALWAYS_AVAILABLE. Preparado por otro chat, empaquetado en zip y verificado aqui de forma independiente antes de aplicar: diff linea por linea de los 3 xlsx contra el estado real del repo (0 discrepancias en las 41 filas existentes), diff del properties.service.ts (una sola linea agregada), y verificacion con el servicio real compilado (189 propiedades totales, San Luis Potosi 44 intacta, 0 IDs duplicados).
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -2200,7 +2200,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -2210,42 +2210,84 @@
           <t>San Luis Potosí 44, Roma Nte., Cuauhtémoc, 06700 Ciudad de México, CDMX, Mexico</t>
         </is>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" s="0" t="n">
         <v>48000</v>
       </c>
-      <c r="D42" t="n">
-        <v>2</v>
-      </c>
-      <c r="E42" t="n">
-        <v>2</v>
-      </c>
-      <c r="F42" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" t="n">
+      <c r="D42" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" s="0" t="inlineStr">
         <is>
           <t>Terraza, Roof garden, Gym</t>
         </is>
       </c>
-      <c r="I42" t="n">
+      <c r="I42" s="0" t="n">
         <v>160</v>
       </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
+      <c r="J42" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K42" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="4" t="n"/>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Tennyson 155, Polanco, Polanco IV Secc, Miguel Hidalgo, 11550 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>68000</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" t="n">
+        <v>5</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Terraza, Jacuzzi</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>235</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="4" t="n"/>

</xml_diff>

<commit_message>
Agregar propiedad #44: Lamartine 136, Polanco, CDMX. 61,000 MXN/mes, 3 recamaras, 3.5 banos, 2 estacionamientos, 210 m2, 6 huespedes (asumido, no confirmado), sin balcon (asumido, no confirmado), pet friendly, amenidad: terraza. 10 fotos + ambos thumbnails de portada. Agregada a ALWAYS_AVAILABLE. IMPORTANTE: el zip venia con un properties.service.ts desactualizado (de antes de marcar Choapan 45/Culiacan 40/Celaya 4/Chicontepec 57 como ocupadas) -- NO se uso ese archivo completo, se aplico solo la linea nueva ('lamartine 136') a mano sobre el archivo real actual, preservando los 4 cambios de disponibilidad mas recientes. Verificado con el servicio real compilado: 190 propiedades, Lamartine correcta, las 4 ocupaciones preservadas, Tennyson 155 intacta, 0 IDs duplicados.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -2245,7 +2245,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -2255,42 +2255,84 @@
           <t>Tennyson 155, Polanco, Polanco IV Secc, Miguel Hidalgo, 11550 Ciudad de México, CDMX, Mexico</t>
         </is>
       </c>
-      <c r="C43" t="n">
+      <c r="C43" s="0" t="n">
         <v>68000</v>
       </c>
-      <c r="D43" t="n">
-        <v>2</v>
-      </c>
-      <c r="E43" t="n">
+      <c r="D43" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="F43" t="n">
-        <v>2</v>
-      </c>
-      <c r="G43" t="n">
+      <c r="F43" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="0" t="inlineStr">
         <is>
           <t>Terraza, Jacuzzi</t>
         </is>
       </c>
-      <c r="I43" t="n">
+      <c r="I43" s="0" t="n">
         <v>235</v>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="4" t="n"/>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Lamartine 136, Polanco, Polanco V Secc, Miguel Hidalgo, 11560 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>61000</v>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" t="n">
+        <v>6</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Terraza</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>210</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="4" t="n"/>

</xml_diff>

<commit_message>
Agregar propiedad #45: Campos Eliseos 100, Polanco, CDMX. 70,000 MXN/mes, 2 recamaras, 2.5 banos, 2 estacionamientos, 160 m2, 4 huespedes, con balcon, pet friendly, amenidades: terraza, gym. 15 fotos + ambos thumbnails de portada. Agregada a ALWAYS_AVAILABLE (confirmado que no colisiona con la propiedad ya existente Campos Eliseos 199, direccion distinta). Preparado por otro chat via zip, verificado aqui de forma independiente: diff limpio de los 3 xlsx contra el estado real (0 discrepancias en las 43 filas existentes), Y IMPORTANTE -- el properties.service.ts del zip estaba basado en una version anterior a la auditoria de esta noche, asi que solo se aplico la linea nueva a mano en vez de reemplazar el archivo completo, preservando los 4 cambios de disponibilidad ocupada mas recientes (Choapan 45, Culiacan 40, Celaya 4, Chicontepec 57). Verificado con el servicio real compilado: 191 propiedades totales, 0 IDs duplicados, Campos Eliseos 199 y Lamartine 136 sin cambios.
</commit_message>
<xml_diff>
--- a/backend/imagenes/CDMX/1/Formato CDMX.xlsx
+++ b/backend/imagenes/CDMX/1/Formato CDMX.xlsx
@@ -2290,7 +2290,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="0" t="inlineStr">
         <is>
           <t>Ciudad de México</t>
         </is>
@@ -2300,42 +2300,84 @@
           <t>Lamartine 136, Polanco, Polanco V Secc, Miguel Hidalgo, 11560 Ciudad de México, CDMX, Mexico</t>
         </is>
       </c>
-      <c r="C44" t="n">
+      <c r="C44" s="0" t="n">
         <v>61000</v>
       </c>
-      <c r="D44" t="n">
+      <c r="D44" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="0" t="n">
         <v>3.5</v>
       </c>
-      <c r="F44" t="n">
-        <v>2</v>
-      </c>
-      <c r="G44" t="n">
+      <c r="F44" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H44" s="0" t="inlineStr">
         <is>
           <t>Terraza</t>
         </is>
       </c>
-      <c r="I44" t="n">
+      <c r="I44" s="0" t="n">
         <v>210</v>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J44" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K44" s="0" t="inlineStr">
         <is>
           <t>si</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="4" t="n"/>
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Campos Elíseos 100, Polanco, Polanco V Secc, Miguel Hidalgo, 11560 Ciudad de México, CDMX, Mexico</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" s="0" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F45" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="H45" s="0" t="inlineStr">
+        <is>
+          <t>Terraza, Gym</t>
+        </is>
+      </c>
+      <c r="I45" s="0" t="n">
+        <v>160</v>
+      </c>
+      <c r="J45" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K45" s="0" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="4" t="n"/>

</xml_diff>